<commit_message>
new asset zinzino added
</commit_message>
<xml_diff>
--- a/Auswertung/Portfolio_Profi_Analyse_B.xlsx
+++ b/Auswertung/Portfolio_Profi_Analyse_B.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Portfolio_Excel\Auswertung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807EA032-166E-4602-AE55-A641D6BFB27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB7FE36-A99C-45A4-8EAE-04C304F8EE69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daten" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId9"/>
+    <pivotCache cacheId="10" r:id="rId9"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9816" uniqueCount="1443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9849" uniqueCount="1448">
   <si>
     <t>datetime</t>
   </si>
@@ -4435,6 +4435,21 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>01a0f3f9-655c-7a49-a2a3-82fe1f75bb85</t>
+  </si>
+  <si>
+    <t>Zinzino</t>
+  </si>
+  <si>
+    <t>SE0002480442</t>
+  </si>
+  <si>
+    <t>Buy trade SE0002480442 ZINZINO AB B, quantity: 8.503401</t>
+  </si>
+  <si>
+    <t>6846f03f-eaef-44a4-bca2-43e995251319</t>
   </si>
 </sst>
 </file>
@@ -4682,7 +4697,92 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Währung" xfId="1" builtinId="4"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="46">
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -4714,13 +4814,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
@@ -4731,6 +4824,24 @@
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
@@ -4749,24 +4860,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="34" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
@@ -11719,9 +11812,9 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Pivot!$A$14:$A$47</c:f>
+              <c:f>Pivot!$A$14:$A$48</c:f>
               <c:multiLvlStrCache>
-                <c:ptCount val="30"/>
+                <c:ptCount val="31"/>
                 <c:lvl>
                   <c:pt idx="0">
                     <c:v>Algorand</c:v>
@@ -11813,6 +11906,9 @@
                   <c:pt idx="29">
                     <c:v>Uranium Energy</c:v>
                   </c:pt>
+                  <c:pt idx="30">
+                    <c:v>Zinzino</c:v>
+                  </c:pt>
                 </c:lvl>
                 <c:lvl>
                   <c:pt idx="0">
@@ -11830,10 +11926,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot!$B$14:$B$47</c:f>
+              <c:f>Pivot!$B$14:$B$48</c:f>
               <c:numCache>
                 <c:formatCode>_("€"* #,##0.00_);_("€"* \(#,##0.00\);_("€"* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="30"/>
+                <c:ptCount val="31"/>
                 <c:pt idx="0">
                   <c:v>17.282800027553129</c:v>
                 </c:pt>
@@ -11923,6 +12019,9 @@
                 </c:pt>
                 <c:pt idx="29">
                   <c:v>516.32673193000005</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>98.044213529999993</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12475,7 +12574,7 @@
                   <c:v>9150.1811199299991</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3633.6654573699998</c:v>
+                  <c:v>3734.68586125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12541,7 +12640,7 @@
                   <c:v>9277.2187277829998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2707.9265223937</c:v>
+                  <c:v>2805.9707359237</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -13315,7 +13414,7 @@
                   <c:v>9277.2187277829998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2707.9265223937</c:v>
+                  <c:v>2805.9707359237</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -15754,7 +15853,7 @@
               <a:cs typeface="Calibri"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t> 14.072,59 € </a:t>
+            <a:t> 14.173,61 € </a:t>
           </a:fld>
           <a:endParaRPr lang="de-DE" sz="2800" b="1">
             <a:ln>
@@ -15844,7 +15943,7 @@
               <a:cs typeface="Calibri"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t> 13.275,56 € </a:t>
+            <a:t> 13.373,60 € </a:t>
           </a:fld>
           <a:endParaRPr lang="de-DE" sz="2800" b="1">
             <a:ln>
@@ -15934,7 +16033,7 @@
               <a:cs typeface="Calibri"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>-797,03 € </a:t>
+            <a:t>-800,00 € </a:t>
           </a:fld>
           <a:endParaRPr lang="de-DE" sz="2800" b="1">
             <a:ln>
@@ -16621,7 +16720,7 @@
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>366,75 €</a:t>
+            <a:t>363,77 €</a:t>
           </a:fld>
           <a:endParaRPr lang="de-DE" sz="1800" b="1">
             <a:ln>
@@ -16711,7 +16810,7 @@
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t>299,81 €</a:t>
+            <a:t>296,84 €</a:t>
           </a:fld>
           <a:endParaRPr lang="de-DE" sz="1800" b="1">
             <a:ln>
@@ -16988,7 +17087,7 @@
               <a:cs typeface="Calibri"/>
             </a:rPr>
             <a:pPr algn="ctr"/>
-            <a:t> 13.275,56 € </a:t>
+            <a:t> 13.373,60 € </a:t>
           </a:fld>
           <a:endParaRPr lang="de-DE" sz="2800" b="1">
             <a:ln>
@@ -17008,13 +17107,13 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Talla Fotsing Roméo" refreshedDate="46295.398773379631" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="62" xr:uid="{AECC3722-4F33-446B-9A76-E2824C46E9CC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Talla Fotsing Roméo" refreshedDate="46295.946661111113" missingItemsLimit="0" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="63" xr:uid="{AECC3722-4F33-446B-9A76-E2824C46E9CC}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:W1048576" sheet="Auswertung"/>
   </cacheSource>
   <cacheFields count="23">
     <cacheField name="Asset" numFmtId="0">
-      <sharedItems containsBlank="1" count="62">
+      <sharedItems containsBlank="1" count="63">
         <s v="Algorand"/>
         <s v="Bayer"/>
         <s v="BP"/>
@@ -17076,6 +17175,7 @@
         <s v="Wizz Air"/>
         <s v="WuXi Biologics"/>
         <s v="XRP"/>
+        <s v="Zinzino"/>
         <m/>
       </sharedItems>
     </cacheField>
@@ -17160,7 +17260,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="62">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="63">
   <r>
     <x v="0"/>
     <x v="0"/>
@@ -18688,6 +18788,31 @@
   </r>
   <r>
     <x v="61"/>
+    <x v="1"/>
+    <s v="SE0002480442"/>
+    <n v="8.5034010000000002"/>
+    <n v="0"/>
+    <n v="8.5034010000000002"/>
+    <n v="100"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="-101"/>
+    <s v="OFFEN"/>
+    <n v="11.88"/>
+    <n v="11.53"/>
+    <n v="-2.9761903500000102"/>
+    <n v="98.044213529999993"/>
+    <n v="101.02040388"/>
+    <n v="-2.946127946127956E-2"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="-2.9557864700000068E-2"/>
+  </r>
+  <r>
+    <x v="62"/>
     <x v="3"/>
     <m/>
     <m/>
@@ -18715,181 +18840,11 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9691FC7-B584-44C9-8056-E4ED1D6024DD}" name="PivotTable11" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
-  <location ref="E3:E4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="23">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item h="1" x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0" numFmtId="44"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="7">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E0769888-D3D4-498F-9981-49DFC80F5D0F}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
-  <location ref="G3:G4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="23">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0" numFmtId="44"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="8">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8E326F01-EA15-4A93-82D4-848E4D2615C7}" name="PivotTable9" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
-  <location ref="J3:J4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="23">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Einkaufswert" fld="15" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="9">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4A41211-FADE-4A81-A35B-B4ED20E62223}" name="PivotTable10" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Assets">
-  <location ref="E13:F17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{223E5646-EA4E-4DBC-8347-0CFCE76D5F19}" name="PivotTable5" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Assets">
+  <location ref="A3:C7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="23">
     <pivotField showAll="0">
-      <items count="63">
+      <items count="64">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -18952,207 +18907,7 @@
         <item x="59"/>
         <item x="60"/>
         <item x="61"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item h="1" x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="10">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="5">
-    <chartFormat chart="3" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="7">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="8">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="9">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="10">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{223E5646-EA4E-4DBC-8347-0CFCE76D5F19}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Assets">
-  <location ref="A3:C7" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="23">
-    <pivotField showAll="0">
-      <items count="63">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="37"/>
-        <item x="38"/>
-        <item x="39"/>
-        <item x="40"/>
-        <item x="41"/>
-        <item x="42"/>
-        <item x="43"/>
-        <item x="44"/>
-        <item x="45"/>
-        <item x="46"/>
-        <item x="47"/>
-        <item x="48"/>
-        <item x="49"/>
-        <item x="50"/>
-        <item x="51"/>
-        <item x="52"/>
-        <item x="53"/>
-        <item x="54"/>
-        <item x="55"/>
-        <item x="56"/>
-        <item x="57"/>
-        <item x="58"/>
-        <item x="59"/>
-        <item x="60"/>
-        <item x="61"/>
+        <item x="62"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -19220,7 +18975,7 @@
     <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="11">
+    <format dxfId="40">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19256,12 +19011,12 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D646C2F3-32F0-4399-B83F-C10E1649A49F}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" preserveFormatting="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="Assets">
-  <location ref="A13:B47" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D646C2F3-32F0-4399-B83F-C10E1649A49F}" name="PivotTable6" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" preserveFormatting="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="Assets">
+  <location ref="A13:B48" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="23">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
-      <items count="63">
+      <items count="64">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -19323,6 +19078,7 @@
         <item x="58"/>
         <item x="59"/>
         <item x="60"/>
+        <item x="62"/>
         <item x="61"/>
         <item t="default"/>
       </items>
@@ -19362,7 +19118,7 @@
     <field x="1"/>
     <field x="0"/>
   </rowFields>
-  <rowItems count="34">
+  <rowItems count="35">
     <i>
       <x/>
     </i>
@@ -19461,6 +19217,9 @@
     </i>
     <i r="1">
       <x v="53"/>
+    </i>
+    <i r="1">
+      <x v="62"/>
     </i>
     <i t="grand">
       <x/>
@@ -20454,8 +20213,124 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1A3F31EA-6894-49F2-AD85-69A514AE323F}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9691FC7-B584-44C9-8056-E4ED1D6024DD}" name="PivotTable11" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+  <location ref="E3:E4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="23">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item h="1" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0" numFmtId="44"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="41">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E0769888-D3D4-498F-9981-49DFC80F5D0F}" name="PivotTable8" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+  <location ref="G3:G4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="23">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0" numFmtId="44"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="42">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1A3F31EA-6894-49F2-AD85-69A514AE323F}" name="PivotTable1" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
   <location ref="L3:L4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="23">
     <pivotField showAll="0"/>
@@ -20500,7 +20375,7 @@
     <dataField name="Verkaufserlöse Gewinn/Verlust" fld="17" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="12">
+    <format dxfId="43">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -20516,12 +20391,66 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{745C1A6C-3C9D-40E8-BB3C-38468AC3798B}" name="PivotTable12" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
-  <location ref="A8:D48" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8E326F01-EA15-4A93-82D4-848E4D2615C7}" name="PivotTable9" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+  <location ref="J3:J4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="23">
-    <pivotField axis="axisRow" subtotalTop="0" showAll="0" insertBlankRow="1" measureFilter="1">
-      <items count="63">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Einkaufswert" fld="15" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="44">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4A41211-FADE-4A81-A35B-B4ED20E62223}" name="PivotTable10" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Assets">
+  <location ref="E13:F17" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="23">
+    <pivotField showAll="0">
+      <items count="64">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -20584,6 +20513,209 @@
         <item x="59"/>
         <item x="60"/>
         <item x="61"/>
+        <item x="62"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item h="1" x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="45">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="5">
+    <chartFormat chart="3" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="10">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{745C1A6C-3C9D-40E8-BB3C-38468AC3798B}" name="PivotTable12" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+  <location ref="A8:D49" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="23">
+    <pivotField axis="axisRow" subtotalTop="0" showAll="0" insertBlankRow="1" measureFilter="1">
+      <items count="64">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item x="50"/>
+        <item x="51"/>
+        <item x="52"/>
+        <item x="53"/>
+        <item x="54"/>
+        <item x="55"/>
+        <item x="56"/>
+        <item x="57"/>
+        <item x="58"/>
+        <item x="59"/>
+        <item x="60"/>
+        <item x="62"/>
+        <item x="61"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -20622,7 +20754,7 @@
     <field x="1"/>
     <field x="0"/>
   </rowFields>
-  <rowItems count="40">
+  <rowItems count="41">
     <i>
       <x/>
     </i>
@@ -20734,6 +20866,9 @@
     <i r="1">
       <x v="53"/>
     </i>
+    <i r="1">
+      <x v="62"/>
+    </i>
     <i t="default">
       <x v="2"/>
     </i>
@@ -20764,10 +20899,10 @@
     <dataField name="Aktueller Wert" fld="14" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="19">
+    <format dxfId="39">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="38">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -20776,7 +20911,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="17">
+    <format dxfId="37">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -20785,7 +20920,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="16">
+    <format dxfId="36">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -20794,7 +20929,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -20803,7 +20938,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="34">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -20812,7 +20947,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="33">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1">
@@ -20855,7 +20990,7 @@
   </pivotTables>
   <data>
     <tabular pivotCacheId="726541802">
-      <items count="62">
+      <items count="63">
         <i x="0" s="1"/>
         <i x="1" s="1"/>
         <i x="2" s="1"/>
@@ -20917,7 +21052,8 @@
         <i x="58" s="1"/>
         <i x="59" s="1"/>
         <i x="60" s="1"/>
-        <i x="61" s="1" nd="1"/>
+        <i x="61" s="1"/>
+        <i x="62" s="1" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -21239,7 +21375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W669"/>
+  <dimension ref="A1:W671"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.85546875" style="32" bestFit="1" customWidth="1"/>
@@ -68763,6 +68899,148 @@
         <v>1442</v>
       </c>
       <c r="W669" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="670" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A670" s="39">
+        <v>46295.930590694399</v>
+      </c>
+      <c r="B670" s="40">
+        <v>46295</v>
+      </c>
+      <c r="C670" t="s">
+        <v>23</v>
+      </c>
+      <c r="D670" t="s">
+        <v>24</v>
+      </c>
+      <c r="E670" t="s">
+        <v>25</v>
+      </c>
+      <c r="F670" t="s">
+        <v>1442</v>
+      </c>
+      <c r="G670" t="s">
+        <v>774</v>
+      </c>
+      <c r="H670" t="s">
+        <v>1442</v>
+      </c>
+      <c r="I670">
+        <v>0</v>
+      </c>
+      <c r="J670">
+        <v>0</v>
+      </c>
+      <c r="K670">
+        <v>101</v>
+      </c>
+      <c r="L670">
+        <v>0</v>
+      </c>
+      <c r="M670">
+        <v>0</v>
+      </c>
+      <c r="N670" t="s">
+        <v>26</v>
+      </c>
+      <c r="O670">
+        <v>0</v>
+      </c>
+      <c r="P670" t="s">
+        <v>1442</v>
+      </c>
+      <c r="Q670">
+        <v>0</v>
+      </c>
+      <c r="R670" t="s">
+        <v>246</v>
+      </c>
+      <c r="S670" t="s">
+        <v>1443</v>
+      </c>
+      <c r="T670" t="s">
+        <v>774</v>
+      </c>
+      <c r="U670" t="s">
+        <v>776</v>
+      </c>
+      <c r="V670" t="s">
+        <v>1442</v>
+      </c>
+      <c r="W670" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="671" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A671" s="39">
+        <v>46295.930676736098</v>
+      </c>
+      <c r="B671" s="40">
+        <v>46295</v>
+      </c>
+      <c r="C671" t="s">
+        <v>23</v>
+      </c>
+      <c r="D671" t="s">
+        <v>30</v>
+      </c>
+      <c r="E671" t="s">
+        <v>31</v>
+      </c>
+      <c r="F671" t="s">
+        <v>32</v>
+      </c>
+      <c r="G671" t="s">
+        <v>1444</v>
+      </c>
+      <c r="H671" t="s">
+        <v>1445</v>
+      </c>
+      <c r="I671">
+        <v>8.5034010000000002</v>
+      </c>
+      <c r="J671">
+        <v>11.76</v>
+      </c>
+      <c r="K671">
+        <v>-100</v>
+      </c>
+      <c r="L671">
+        <v>-1</v>
+      </c>
+      <c r="M671">
+        <v>0</v>
+      </c>
+      <c r="N671" t="s">
+        <v>26</v>
+      </c>
+      <c r="O671">
+        <v>0</v>
+      </c>
+      <c r="P671" t="s">
+        <v>1442</v>
+      </c>
+      <c r="Q671">
+        <v>0</v>
+      </c>
+      <c r="R671" t="s">
+        <v>1446</v>
+      </c>
+      <c r="S671" t="s">
+        <v>1447</v>
+      </c>
+      <c r="T671" t="s">
+        <v>1442</v>
+      </c>
+      <c r="U671" t="s">
+        <v>1442</v>
+      </c>
+      <c r="V671" t="s">
+        <v>1442</v>
+      </c>
+      <c r="W671" t="s">
         <v>1442</v>
       </c>
     </row>
@@ -71973,7 +72251,7 @@
         <v>1.3543989999999999</v>
       </c>
       <c r="F34" s="5">
-        <f t="shared" ref="F34:F62" si="10">D34-E34</f>
+        <f t="shared" ref="F34:F63" si="10">D34-E34</f>
         <v>0</v>
       </c>
       <c r="G34" s="6">
@@ -71989,11 +72267,11 @@
         <v>4</v>
       </c>
       <c r="J34" s="6">
-        <f t="shared" ref="J34:J62" si="11">H34-G34-I34</f>
+        <f t="shared" ref="J34:J63" si="11">H34-G34-I34</f>
         <v>5.1899999999999977</v>
       </c>
       <c r="K34" s="5" t="str">
-        <f t="shared" ref="K34:K62" si="12">IF(F34&gt;0,"OFFEN","GESCHLOSSEN")</f>
+        <f t="shared" ref="K34:K63" si="12">IF(F34&gt;0,"OFFEN","GESCHLOSSEN")</f>
         <v>GESCHLOSSEN</v>
       </c>
       <c r="L34">
@@ -72003,7 +72281,7 @@
         <v>0</v>
       </c>
       <c r="N34" s="21">
-        <f t="shared" ref="N34:N62" si="13">IF(K34="GESCHLOSSEN",
+        <f t="shared" ref="N34:N63" si="13">IF(K34="GESCHLOSSEN",
 0,
 IF(K34="OFFEN",
 ((M34*F34)-(L34*F34)),
@@ -72011,15 +72289,15 @@
         <v>0</v>
       </c>
       <c r="O34" s="6">
-        <f t="shared" ref="O34:O62" si="14">IF(F34&gt;0,F34*M34,0)</f>
+        <f t="shared" ref="O34:O63" si="14">IF(F34&gt;0,F34*M34,0)</f>
         <v>0</v>
       </c>
       <c r="P34" s="6">
-        <f t="shared" ref="P34:P62" si="15">IF(F34&gt;0,F34*L34,0)</f>
+        <f t="shared" ref="P34:P63" si="15">IF(F34&gt;0,F34*L34,0)</f>
         <v>0</v>
       </c>
       <c r="Q34" s="7">
-        <f t="shared" ref="Q34:Q62" si="16">IF(K34="GESCHLOSSEN",
+        <f t="shared" ref="Q34:Q63" si="16">IF(K34="GESCHLOSSEN",
 0,
 IF(K34="OFFEN",
 (N34/(L34*F34))))</f>
@@ -72037,7 +72315,7 @@
         <v>5.1999999999999975</v>
       </c>
       <c r="S34" s="6">
-        <f t="shared" ref="S34:S62" si="17">IF(E34=0,
+        <f t="shared" ref="S34:S63" si="17">IF(E34=0,
 0,
 (G34-(F34*L34))+I34
 )</f>
@@ -72052,11 +72330,11 @@
         <v>2</v>
       </c>
       <c r="V34" s="7">
-        <f t="shared" ref="V34:V62" si="18">IF(S34&gt;0,R34/S34,0)</f>
+        <f t="shared" ref="V34:V63" si="18">IF(S34&gt;0,R34/S34,0)</f>
         <v>2.5999999999999988E-2</v>
       </c>
       <c r="W34" s="7">
-        <f t="shared" ref="W34:W62" si="19">IF(K34="GESCHLOSSEN",
+        <f t="shared" ref="W34:W63" si="19">IF(K34="GESCHLOSSEN",
 J34/(G34+I34),
 IF(K34="OFFEN",
 ((H34+M34*F34)-G34-I34)/G34,
@@ -74750,6 +75028,102 @@
       <c r="W62" s="7">
         <f t="shared" si="19"/>
         <v>-9.1908819339886864E-3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A63" s="9" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C63" s="5" t="s">
+        <v>1445</v>
+      </c>
+      <c r="D63" s="5">
+        <f>SUMIFS(Daten!I:I,Daten!H:H,C63,Daten!E:E,"BUY")</f>
+        <v>8.5034010000000002</v>
+      </c>
+      <c r="E63" s="5">
+        <f>-SUMIFS(Daten!I:I,Daten!H:H,C63,Daten!E:E,"SELL")</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="5">
+        <f t="shared" si="10"/>
+        <v>8.5034010000000002</v>
+      </c>
+      <c r="G63" s="6">
+        <f>-SUMIFS(Daten!K:K,Daten!H:H,C63,Daten!E:E,"BUY")</f>
+        <v>100</v>
+      </c>
+      <c r="H63" s="6">
+        <f>SUMIFS(Daten!K:K,Daten!H:H,C63,Daten!E:E,"SELL")</f>
+        <v>0</v>
+      </c>
+      <c r="I63" s="6">
+        <f>SUMIFS(Daten!L:L,Daten!H:H,C63)*-1</f>
+        <v>1</v>
+      </c>
+      <c r="J63" s="6">
+        <f t="shared" si="11"/>
+        <v>-101</v>
+      </c>
+      <c r="K63" s="5" t="str">
+        <f t="shared" si="12"/>
+        <v>OFFEN</v>
+      </c>
+      <c r="L63" s="21">
+        <v>11.88</v>
+      </c>
+      <c r="M63" s="21">
+        <v>11.53</v>
+      </c>
+      <c r="N63" s="21">
+        <f t="shared" si="13"/>
+        <v>-2.9761903500000102</v>
+      </c>
+      <c r="O63" s="6">
+        <f t="shared" si="14"/>
+        <v>98.044213529999993</v>
+      </c>
+      <c r="P63" s="6">
+        <f t="shared" si="15"/>
+        <v>101.02040388</v>
+      </c>
+      <c r="Q63" s="7">
+        <f t="shared" si="16"/>
+        <v>-2.946127946127956E-2</v>
+      </c>
+      <c r="R63" s="6">
+        <f>IF(K63="GESCHLOSSEN",
+H63-G63-I63 + SUMIFS(Daten!K:K,Daten!H:H,C63,Daten!E:E,"DIVIDEND"),
+IF(K63="OFFEN",
+IF(E63=0,
+0,
+H63+SUMIFS(Daten!K:K,Daten!H:H,C63,Daten!E:E,"DIVIDEND")-(G63-(F63*L63))-I63
+),
+""))</f>
+        <v>0</v>
+      </c>
+      <c r="S63" s="6">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="T63" s="26">
+        <f>COUNTIFS(Daten!H:H,C63,Daten!E:E,"BUY",Daten!L:L,"&lt;0")</f>
+        <v>1</v>
+      </c>
+      <c r="U63" s="26">
+        <f>COUNTIFS(Daten!H:H,C63,Daten!E:E,"SELL",Daten!L:L,"&lt;0")</f>
+        <v>0</v>
+      </c>
+      <c r="V63" s="7">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="W63" s="7">
+        <f t="shared" si="19"/>
+        <v>-2.9557864700000068E-2</v>
       </c>
     </row>
     <row r="76" spans="28:29" x14ac:dyDescent="0.25">
@@ -74833,29 +75207,29 @@
     <sortCondition ref="A2:A86"/>
   </sortState>
   <conditionalFormatting sqref="N2:N1048576">
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="8" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="9" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="11" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:R1048576">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="32" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V2:W1048576">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="30" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -74891,7 +75265,7 @@
       </c>
       <c r="B3" s="11">
         <f>COUNTA(Auswertung!A:A) - 1</f>
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C3" s="23">
         <f>IF(ABS(B3)&gt;0,B3/B3,0)</f>
@@ -74904,11 +75278,11 @@
       </c>
       <c r="B4" s="11">
         <f>COUNTIFS(Auswertung!B:B,"STOCK")</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" s="23">
         <f>IF(ABS(B3)&gt;0,B4/B3,0)</f>
-        <v>0.62295081967213117</v>
+        <v>0.62903225806451613</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -74921,7 +75295,7 @@
       </c>
       <c r="C5" s="23">
         <f>IF(ABS(B3)&gt;0,B5/B3,0)</f>
-        <v>0.22950819672131148</v>
+        <v>0.22580645161290322</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -74934,7 +75308,7 @@
       </c>
       <c r="C6" s="23">
         <f>IF(ABS(B3)&gt;0,B6/B3,0)</f>
-        <v>0.14754098360655737</v>
+        <v>0.14516129032258066</v>
       </c>
     </row>
     <row r="7" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -74947,7 +75321,7 @@
       </c>
       <c r="B8" s="11">
         <f>COUNTIFS(Auswertung!K:K,"OFFEN")</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="23">
         <f>IF(ABS(B8)&gt;0,B8/B8,0)</f>
@@ -74960,11 +75334,11 @@
       </c>
       <c r="B9" s="11">
         <f>COUNTIFS(Auswertung!B:B,"STOCK",Auswertung!K:K,"OFFEN")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="23">
         <f>IF(ABS(B8)&gt;0,B9/B8,0)</f>
-        <v>0.26666666666666666</v>
+        <v>0.29032258064516131</v>
       </c>
     </row>
     <row r="10" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -74977,7 +75351,7 @@
       </c>
       <c r="C10" s="23">
         <f>IF(ABS(B8)&gt;0,B10/B8,0)</f>
-        <v>0.43333333333333335</v>
+        <v>0.41935483870967744</v>
       </c>
     </row>
     <row r="11" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -74990,7 +75364,7 @@
       </c>
       <c r="C11" s="23">
         <f>IF(ABS(B8)&gt;0,B11/B8,0)</f>
-        <v>0.3</v>
+        <v>0.29032258064516131</v>
       </c>
     </row>
     <row r="12" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75043,11 +75417,11 @@
       </c>
       <c r="B18" s="14">
         <f>SUM(Auswertung!G:G)-SUMIFS(Daten!L:L,Daten!E:E,"BUY")</f>
-        <v>24703.460000000003</v>
+        <v>24804.460000000003</v>
       </c>
       <c r="D18" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!E:E,"BUY")-SUMIFS(Daten!L:L,Daten!E:E,"BUY")</f>
-        <v>24703.460000000003</v>
+        <v>24804.460000000003</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75056,15 +75430,15 @@
       </c>
       <c r="B19" s="14">
         <f>SUMIFS(Auswertung!G:G,Auswertung!B:B,"STOCK")+SUMIFS(Auswertung!G:G,Auswertung!B:B,"FUND")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"STOCK")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"FUND")</f>
-        <v>22621.809999999998</v>
+        <v>22722.809999999998</v>
       </c>
       <c r="C19" s="23">
         <f>IF(ABS(B18)&gt;0,B19/B18,0)</f>
-        <v>0.91573447606124792</v>
+        <v>0.91607759249747811</v>
       </c>
       <c r="D19" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"STOCK",Daten!E:E,"BUY")-SUMIFS(Daten!K:K,Daten!F:F,"FUND",Daten!E:E,"BUY")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"STOCK")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"FUND")</f>
-        <v>22621.809999999998</v>
+        <v>22722.809999999998</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75073,15 +75447,15 @@
       </c>
       <c r="B20" s="14">
         <f>SUMIFS(Auswertung!G:G,Auswertung!B:B,"STOCK")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"STOCK")</f>
-        <v>12969.64</v>
+        <v>13070.64</v>
       </c>
       <c r="C20" s="23">
         <f>IF(ABS(B18)&gt;0,B20/B18,0)</f>
-        <v>0.52501309533158502</v>
+        <v>0.52694716998475266</v>
       </c>
       <c r="D20" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"STOCK",Daten!E:E,"BUY")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"STOCK")</f>
-        <v>12969.64</v>
+        <v>13070.64</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75094,7 +75468,7 @@
       </c>
       <c r="C21" s="23">
         <f>IF(ABS(B18)&gt;0,B21/B18,0)</f>
-        <v>0.39072138072966295</v>
+        <v>0.3891304225127255</v>
       </c>
       <c r="D21" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"FUND",Daten!E:E,"BUY")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"FUND")</f>
@@ -75111,7 +75485,7 @@
       </c>
       <c r="C22" s="23">
         <f>IF(ABS(B18)&gt;0,B22/B18,0)</f>
-        <v>8.4265523938751891E-2</v>
+        <v>8.3922407502521723E-2</v>
       </c>
       <c r="D22" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"CRYPTO",Daten!E:E,"BUY")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"CRYPTO")</f>
@@ -75130,12 +75504,12 @@
       </c>
       <c r="B24" s="14">
         <f>SUM(Auswertung!G:G)</f>
-        <v>24485.460000000003</v>
+        <v>24585.460000000003</v>
       </c>
       <c r="C24" s="23"/>
       <c r="D24" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!E:E,"BUY")</f>
-        <v>24485.460000000003</v>
+        <v>24585.460000000003</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75144,15 +75518,15 @@
       </c>
       <c r="B25" s="14">
         <f>SUMIFS(Auswertung!G:G,Auswertung!B:B,"STOCK")+SUMIFS(Auswertung!G:G,Auswertung!B:B,"FUND")</f>
-        <v>22442.809999999998</v>
+        <v>22542.809999999998</v>
       </c>
       <c r="C25" s="23">
         <f>IF(ABS(B24)&gt;0,B25/B24,0)</f>
-        <v>0.91657702162834576</v>
+        <v>0.91691633998306299</v>
       </c>
       <c r="D25" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"STOCK",Daten!E:E,"BUY")-SUMIFS(Daten!K:K,Daten!F:F,"FUND",Daten!E:E,"BUY")</f>
-        <v>22442.809999999998</v>
+        <v>22542.809999999998</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75161,15 +75535,15 @@
       </c>
       <c r="B26" s="14">
         <f>SUMIFS(Auswertung!G:G,Auswertung!B:B,"STOCK")</f>
-        <v>12842.64</v>
+        <v>12942.64</v>
       </c>
       <c r="C26" s="23">
         <f>IF(ABS(B24)&gt;0,B26/B24,0)</f>
-        <v>0.52450066284235619</v>
+        <v>0.52643473012097386</v>
       </c>
       <c r="D26" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"STOCK",Daten!E:E,"BUY")</f>
-        <v>12842.64</v>
+        <v>12942.64</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75182,7 +75556,7 @@
       </c>
       <c r="C27" s="23">
         <f>IF(ABS(B24)&gt;0,B27/B24,0)</f>
-        <v>0.39207635878598968</v>
+        <v>0.39048160986208919</v>
       </c>
       <c r="D27" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"FUND",Daten!E:E,"BUY")</f>
@@ -75199,7 +75573,7 @@
       </c>
       <c r="C28" s="23">
         <f>IF(ABS(B24)&gt;0,B28/B24,0)</f>
-        <v>8.3422978371654036E-2</v>
+        <v>8.3083660016936831E-2</v>
       </c>
       <c r="D28" s="22">
         <f>-SUMIFS(Daten!K:K,Daten!F:F,"CRYPTO",Daten!E:E,"BUY")</f>
@@ -75391,11 +75765,11 @@
       </c>
       <c r="B42" s="14">
         <f>SUM(Auswertung!I:I)</f>
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C42" s="22">
         <f>-SUM(Daten!L:L)</f>
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D42" s="23"/>
     </row>
@@ -75405,15 +75779,15 @@
       </c>
       <c r="B43" s="14">
         <f>SUMIFS(Auswertung!I:I,Auswertung!B:B,"STOCK")+SUMIFS(Auswertung!I:I,Auswertung!B:B,"FUND")</f>
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C43" s="22">
         <f xml:space="preserve"> -SUMIFS(Daten!L:L,Daten!F:F,"STOCK")-SUMIFS(Daten!L:L,Daten!F:F,"FUND")</f>
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D43" s="23">
         <f>IF(ABS(C42)&gt;0,C43/C42,0)</f>
-        <v>0.85357142857142854</v>
+        <v>0.85409252669039148</v>
       </c>
     </row>
     <row r="44" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75422,15 +75796,15 @@
       </c>
       <c r="B44" s="14">
         <f>SUMIFS(Auswertung!I:I,Auswertung!B:B,"STOCK")</f>
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C44" s="22">
         <f xml:space="preserve"> -SUMIFS(Daten!L:L,Daten!F:F,"STOCK")</f>
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D44" s="23">
         <f>IF(ABS(C42)&gt;0,C44/C42,0)</f>
-        <v>0.66428571428571426</v>
+        <v>0.66548042704626331</v>
       </c>
     </row>
     <row r="45" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75447,7 +75821,7 @@
       </c>
       <c r="D45" s="23">
         <f>IF(ABS(C42)&gt;0,C45/C42,0)</f>
-        <v>0.18928571428571428</v>
+        <v>0.18861209964412812</v>
       </c>
     </row>
     <row r="46" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75464,7 +75838,7 @@
       </c>
       <c r="D46" s="23">
         <f>IF(ABS(C42)&gt;0,C46/C42,0)</f>
-        <v>0.14642857142857144</v>
+        <v>0.14590747330960854</v>
       </c>
     </row>
     <row r="47" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75477,7 +75851,7 @@
       </c>
       <c r="B48" s="14">
         <f xml:space="preserve"> -SUMIFS(Daten!L:L,Daten!E:E,"BUY")</f>
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="49" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75486,11 +75860,11 @@
       </c>
       <c r="B49" s="14">
         <f xml:space="preserve"> -SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"STOCK")-SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"FUND")</f>
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C49" s="23">
         <f>IF(ABS(B48)&gt;0,B49/B48,0)</f>
-        <v>0.82110091743119262</v>
+        <v>0.82191780821917804</v>
       </c>
     </row>
     <row r="50" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75499,11 +75873,11 @@
       </c>
       <c r="B50" s="14">
         <f xml:space="preserve"> -SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"STOCK")</f>
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C50" s="23">
         <f>IF(ABS(B48)&gt;0,B50/B48,0)</f>
-        <v>0.58256880733944949</v>
+        <v>0.58447488584474883</v>
       </c>
     </row>
     <row r="51" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75516,7 +75890,7 @@
       </c>
       <c r="C51" s="23">
         <f>IF(ABS(B48)&gt;0,B51/B48,0)</f>
-        <v>0.23853211009174313</v>
+        <v>0.23744292237442921</v>
       </c>
     </row>
     <row r="52" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75529,7 +75903,7 @@
       </c>
       <c r="C52" s="23">
         <f>IF(ABS(B48)&gt;0,B52/B48,0)</f>
-        <v>0.17889908256880735</v>
+        <v>0.17808219178082191</v>
       </c>
     </row>
     <row r="53" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75609,7 +75983,7 @@
       </c>
       <c r="B60" s="29">
         <f xml:space="preserve"> SUM(Auswertung!T:T)</f>
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C60" s="23"/>
     </row>
@@ -75619,11 +75993,11 @@
       </c>
       <c r="B61" s="29">
         <f xml:space="preserve"> SUMIFS(Auswertung!T:T,Auswertung!B:B,"STOCK")+SUMIFS(Auswertung!T:T,Auswertung!B:B,"FUND")</f>
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C61" s="23">
         <f>IF(ABS(B60)&gt;0,B61/B60,0)</f>
-        <v>0.82110091743119262</v>
+        <v>0.82191780821917804</v>
       </c>
     </row>
     <row r="62" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75632,11 +76006,11 @@
       </c>
       <c r="B62" s="29">
         <f>SUMIFS(Auswertung!T:T,Auswertung!B:B,"STOCK")</f>
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C62" s="23">
         <f>IF(ABS(B60)&gt;0,B62/B60,0)</f>
-        <v>0.58256880733944949</v>
+        <v>0.58447488584474883</v>
       </c>
     </row>
     <row r="63" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75649,7 +76023,7 @@
       </c>
       <c r="C63" s="23">
         <f>IF(ABS(B60)&gt;0,B63/B60,0)</f>
-        <v>0.23853211009174313</v>
+        <v>0.23744292237442921</v>
       </c>
     </row>
     <row r="64" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75662,7 +76036,7 @@
       </c>
       <c r="C64" s="23">
         <f>IF(ABS(B60)&gt;0,B64/B60,0)</f>
-        <v>0.17889908256880735</v>
+        <v>0.17808219178082191</v>
       </c>
     </row>
     <row r="65" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75742,7 +76116,7 @@
       </c>
       <c r="B72" s="14">
         <f>SUM(Auswertung!J:J)</f>
-        <v>-12912.58</v>
+        <v>-13013.58</v>
       </c>
     </row>
     <row r="73" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75751,11 +76125,11 @@
       </c>
       <c r="B73" s="14">
         <f>SUMIFS(Auswertung!J:J,Auswertung!B:B,"STOCK") + SUMIFS(Auswertung!J:J,Auswertung!B:B,"FUND")</f>
-        <v>-11689.49</v>
+        <v>-11790.49</v>
       </c>
       <c r="C73" s="23">
         <f>IF(ABS(B72)&gt;0,B73/B72,0)</f>
-        <v>0.90527919284914404</v>
+        <v>0.90601433272012777</v>
       </c>
     </row>
     <row r="74" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75764,11 +76138,11 @@
       </c>
       <c r="B74" s="14">
         <f>SUMIFS(Auswertung!J:J,Auswertung!B:B,"STOCK")</f>
-        <v>-2542.9299999999998</v>
+        <v>-2643.93</v>
       </c>
       <c r="C74" s="23">
         <f>IF(ABS(B72)&gt;0,B74/B72,0)</f>
-        <v>0.19693430747379687</v>
+        <v>0.20316699939601554</v>
       </c>
     </row>
     <row r="75" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75781,7 +76155,7 @@
       </c>
       <c r="C75" s="23">
         <f>IF(ABS(B72)&gt;0,B75/B72,0)</f>
-        <v>0.70834488537534712</v>
+        <v>0.7028473333241122</v>
       </c>
     </row>
     <row r="76" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75794,7 +76168,7 @@
       </c>
       <c r="C76" s="23">
         <f>IF(ABS(B72)&gt;0,B76/B72,0)</f>
-        <v>9.4720807150855985E-2</v>
+        <v>9.3985667279872245E-2</v>
       </c>
     </row>
     <row r="77" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75930,7 +76304,7 @@
       </c>
       <c r="B91" s="14">
         <f>SUMIFS(Auswertung!O:O,Auswertung!K:K,"OFFEN")</f>
-        <v>13275.558198955154</v>
+        <v>13373.602412485154</v>
       </c>
     </row>
     <row r="92" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75940,11 +76314,11 @@
       <c r="B92" s="14">
         <f>SUMIFS(Auswertung!O:O,Auswertung!K:K,"OFFEN",Auswertung!B:B,"STOCK")
 +SUMIFS(Auswertung!O:O,Auswertung!K:K,"OFFEN",Auswertung!B:B,"FUND")</f>
-        <v>11985.1452501767</v>
+        <v>12083.1894637067</v>
       </c>
       <c r="C92" s="23">
         <f>IF(ABS(B91)&gt;0,B92/B91,0)</f>
-        <v>0.90279783874699782</v>
+        <v>0.90351044475692155</v>
       </c>
     </row>
     <row r="93" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75953,11 +76327,11 @@
       </c>
       <c r="B93" s="14">
         <f>SUMIFS(Auswertung!O:O,Auswertung!K:K,"OFFEN",Auswertung!B:B,"STOCK")</f>
-        <v>2707.9265223937</v>
+        <v>2805.9707359237</v>
       </c>
       <c r="C93" s="23">
         <f>IF(ABS(B91)&gt;0,B93/B91,0)</f>
-        <v>0.20397835494456468</v>
+        <v>0.20981412856300696</v>
       </c>
     </row>
     <row r="94" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75970,7 +76344,7 @@
       </c>
       <c r="C94" s="23">
         <f>IF(ABS(B91)&gt;0,B94/B91,0)</f>
-        <v>0.69881948380243319</v>
+        <v>0.69369631619391459</v>
       </c>
     </row>
     <row r="95" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -75983,7 +76357,7 @@
       </c>
       <c r="C95" s="23">
         <f>IF(ABS(B91)&gt;0,B95/B91,0)</f>
-        <v>9.7202161253002725E-2</v>
+        <v>9.6489555243079034E-2</v>
       </c>
     </row>
     <row r="96" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76000,7 +76374,7 @@
 + SUMIFS(Daten!K:K,Daten!E:E,"GIFT")
 + SUMIFS(Daten!K:K,Daten!E:E,"DIVIDEND")
 + SUMIFS(Daten!K:K,Daten!E:E,"CUSTOMER_INPAYMENT")</f>
-        <v>22468.14</v>
+        <v>22569.14</v>
       </c>
     </row>
     <row r="98" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76022,7 +76396,7 @@
       </c>
       <c r="B100" s="14">
         <f>SUMIFS(Daten!K:K,Daten!E:E,"BUY")+SUMIFS(Daten!L:L,Daten!E:E,"BUY")</f>
-        <v>-24703.460000000003</v>
+        <v>-24804.460000000003</v>
       </c>
     </row>
     <row r="101" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76031,11 +76405,11 @@
       </c>
       <c r="B101" s="14">
         <f>SUMIFS(Daten!K:K,Daten!E:E,"BUY",Daten!F:F,"STOCK")+SUMIFS(Daten!L:L,Daten!E:E,"BUY",Daten!F:F,"STOCK")</f>
-        <v>-12969.64</v>
+        <v>-13070.64</v>
       </c>
       <c r="C101" s="23">
         <f>IF(ABS(B100)&gt;0,B101/B100,0)</f>
-        <v>0.52501309533158502</v>
+        <v>0.52694716998475266</v>
       </c>
     </row>
     <row r="102" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76048,7 +76422,7 @@
       </c>
       <c r="C102" s="23">
         <f>IF(ABS(B100)&gt;0,B102/B100,0)</f>
-        <v>0.39072138072966284</v>
+        <v>0.38913042251272539</v>
       </c>
     </row>
     <row r="103" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76061,7 +76435,7 @@
       </c>
       <c r="C103" s="23">
         <f>IF(ABS(B100)&gt;0,B103/B100,0)</f>
-        <v>8.4265523938751891E-2</v>
+        <v>8.3922407502521723E-2</v>
       </c>
     </row>
     <row r="104" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76126,7 +76500,7 @@
       </c>
       <c r="B110" s="14">
         <f>SUMIFS(Auswertung!P:P,Auswertung!K:K,"OFFEN")</f>
-        <v>14072.586580620899</v>
+        <v>14173.606984500899</v>
       </c>
     </row>
     <row r="111" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76136,11 +76510,11 @@
       <c r="B111" s="14">
         <f>SUMIFS(Auswertung!P:P,Auswertung!K:K,"OFFEN",Auswertung!B:B,"STOCK")
 +SUMIFS(Auswertung!P:P,Auswertung!K:K,"OFFEN",Auswertung!B:B,"FUND")</f>
-        <v>12783.846577299999</v>
+        <v>12884.866981179999</v>
       </c>
       <c r="C111" s="23">
         <f>IF(ABS(B110)&gt;0,B111/B110,0)</f>
-        <v>0.90842195242944179</v>
+        <v>0.90907466217102251</v>
       </c>
     </row>
     <row r="112" spans="1:3" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76149,11 +76523,11 @@
       </c>
       <c r="B112" s="14">
         <f>SUMIFS(Auswertung!P:P,Auswertung!K:K,"OFFEN",Auswertung!B:B,"STOCK")</f>
-        <v>3633.6654573699998</v>
+        <v>3734.68586125</v>
       </c>
       <c r="C112" s="23">
         <f>IF(ABS(B110)&gt;0,B112/B110,0)</f>
-        <v>0.25820878319369189</v>
+        <v>0.26349579647114163</v>
       </c>
     </row>
     <row r="113" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76166,7 +76540,7 @@
       </c>
       <c r="C113" s="23">
         <f>IF(ABS(B110)&gt;0,B113/B110,0)</f>
-        <v>0.6502131692357499</v>
+        <v>0.64557886569988088</v>
       </c>
     </row>
     <row r="114" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76179,7 +76553,7 @@
       </c>
       <c r="C114" s="23">
         <f>IF(ABS(B110)&gt;0,B114/B110,0)</f>
-        <v>9.1578047570558235E-2</v>
+        <v>9.0925337828977562E-2</v>
       </c>
     </row>
     <row r="115" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76192,7 +76566,7 @@
       </c>
       <c r="B116" s="14">
         <f>SUMIFS(Auswertung!N:N,Auswertung!N:N,"&lt;0",Auswertung!K:K,"OFFEN")</f>
-        <v>-1488.4504453027992</v>
+        <v>-1491.4266356527992</v>
       </c>
       <c r="C116" s="23"/>
     </row>
@@ -76203,11 +76577,11 @@
       <c r="B117" s="14">
         <f>SUMIFS(Auswertung!N:N,Auswertung!N:N,"&lt;0",Auswertung!B:B,"STOCK",Auswertung!K:K,"OFFEN")
 +SUMIFS(Auswertung!N:N,Auswertung!N:N,"&lt;0",Auswertung!B:B,"FUND",Auswertung!K:K,"OFFEN")</f>
-        <v>-1397.4843192233002</v>
+        <v>-1400.4605095733002</v>
       </c>
       <c r="C117" s="23">
         <f>IF(ABS(B116)&gt;0,B117/B116,0)</f>
-        <v>0.93888535129498818</v>
+        <v>0.93900730756381923</v>
       </c>
     </row>
     <row r="118" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76216,11 +76590,11 @@
       </c>
       <c r="B118" s="14">
         <f>SUMIFS(Auswertung!N:N,Auswertung!N:N,"&lt;0",Auswertung!B:B,"STOCK",Auswertung!K:K,"OFFEN")</f>
-        <v>-934.93579478930008</v>
+        <v>-937.9119851393001</v>
       </c>
       <c r="C118" s="23">
         <f>IF(ABS(B116)&gt;0,B118/B116,0)</f>
-        <v>0.62812692067763387</v>
+        <v>0.62886900550007607</v>
       </c>
     </row>
     <row r="119" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76233,7 +76607,7 @@
       </c>
       <c r="C119" s="23">
         <f>IF(ABS(B116)&gt;0,B119/B116,0)</f>
-        <v>0.31075843061735436</v>
+        <v>0.31013830206374321</v>
       </c>
     </row>
     <row r="120" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76246,7 +76620,7 @@
       </c>
       <c r="C120" s="23">
         <f>IF(ABS(B116)&gt;0,B120/B116,0)</f>
-        <v>6.1114648705011973E-2</v>
+        <v>6.0992692436180898E-2</v>
       </c>
     </row>
     <row r="121" spans="1:4" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76326,15 +76700,15 @@
       </c>
       <c r="B128" s="14">
         <f>SUMIFS(Auswertung!N:N,Auswertung!K:K,"OFFEN")</f>
-        <v>-797.02838166573952</v>
+        <v>-800.00457201573954</v>
       </c>
       <c r="C128" s="22">
         <f>B91-B110</f>
-        <v>-797.02838166574475</v>
+        <v>-800.004572015745</v>
       </c>
       <c r="D128" s="22">
         <f>B116+B122</f>
-        <v>-797.02838166573906</v>
+        <v>-800.00457201573909</v>
       </c>
     </row>
     <row r="129" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76344,19 +76718,19 @@
       <c r="B129" s="14">
         <f>SUMIFS(Auswertung!N:N,Auswertung!B:B,"STOCK",Auswertung!K:K,"OFFEN")
 +SUMIFS(Auswertung!N:N,Auswertung!B:B,"FUND",Auswertung!K:K,"OFFEN")</f>
-        <v>-798.70132712330042</v>
+        <v>-801.67751747330044</v>
       </c>
       <c r="C129" s="22">
         <f>B92-B111</f>
-        <v>-798.70132712329905</v>
+        <v>-801.6775174732993</v>
       </c>
       <c r="D129" s="22">
         <f>B117+B123</f>
-        <v>-798.70132712330053</v>
+        <v>-801.67751747330055</v>
       </c>
       <c r="E129" s="23">
         <f>IF(ABS(B128)&gt;0,B129/B128,0)</f>
-        <v>1.0020989785257892</v>
+        <v>1.0020911698708741</v>
       </c>
     </row>
     <row r="130" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76365,19 +76739,19 @@
       </c>
       <c r="B130" s="14">
         <f>SUMIFS(Auswertung!N:N,Auswertung!B:B,"STOCK",Auswertung!K:K,"OFFEN")</f>
-        <v>-925.73893497630002</v>
+        <v>-928.71512532630004</v>
       </c>
       <c r="C130" s="22">
         <f>B93-B112</f>
-        <v>-925.73893497629979</v>
+        <v>-928.71512532630004</v>
       </c>
       <c r="D130" s="22">
         <f>B118+B124</f>
-        <v>-925.73893497630013</v>
+        <v>-928.71512532630015</v>
       </c>
       <c r="E130" s="23">
         <f>IF(ABS(B128)&gt;0,B130/B128,0)</f>
-        <v>1.1614880426736667</v>
+        <v>1.1608872721642749</v>
       </c>
     </row>
     <row r="131" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76398,7 +76772,7 @@
       </c>
       <c r="E131" s="23">
         <f>IF(ABS(B128)&gt;0,B131/B128,0)</f>
-        <v>-0.15938906414787749</v>
+        <v>-0.1587961022934006</v>
       </c>
     </row>
     <row r="132" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76419,7 +76793,7 @@
       </c>
       <c r="E132" s="23">
         <f>IF(ABS(B128)&gt;0,B132/B128,0)</f>
-        <v>-2.0989785257895448E-3</v>
+        <v>-2.0911698708745209E-3</v>
       </c>
     </row>
     <row r="133" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76434,7 +76808,7 @@
       </c>
       <c r="B134" s="14">
         <f>B78+B128</f>
-        <v>366.74522646426021</v>
+        <v>363.76903611426019</v>
       </c>
       <c r="C134" s="22"/>
       <c r="D134" s="22"/>
@@ -76445,7 +76819,7 @@
       </c>
       <c r="B135" s="14">
         <f>B79+B129</f>
-        <v>299.81228100669932</v>
+        <v>296.8360906566993</v>
       </c>
       <c r="C135" s="22"/>
       <c r="D135" s="22"/>
@@ -76471,7 +76845,7 @@
       </c>
       <c r="B138" s="14">
         <f>B72+B91</f>
-        <v>362.97819895515386</v>
+        <v>360.02241248515384</v>
       </c>
       <c r="C138" s="22"/>
     </row>
@@ -76481,7 +76855,7 @@
       </c>
       <c r="B139" s="14">
         <f>B73+B92</f>
-        <v>295.65525017670006</v>
+        <v>292.69946370670004</v>
       </c>
       <c r="C139" s="22"/>
       <c r="D139" s="22"/>
@@ -76506,11 +76880,11 @@
       </c>
       <c r="B142" s="15">
         <f>IF(ABS(B72)&gt;0,-B138/B72,0)</f>
-        <v>2.8110431761518912E-2</v>
+        <v>2.7665132306802113E-2</v>
       </c>
       <c r="C142" s="23">
         <f>IF(ABS(B72)&gt;0,-B134/B72,0)</f>
-        <v>2.8402164901534799E-2</v>
+        <v>2.7953033378536898E-2</v>
       </c>
     </row>
     <row r="143" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76519,11 +76893,11 @@
       </c>
       <c r="B143" s="15">
         <f>IF(ABS(B73)&gt;0,-B139/B73,0)</f>
-        <v>2.529239942689545E-2</v>
+        <v>2.4825046601684921E-2</v>
       </c>
       <c r="C143" s="23">
         <f>IF(ABS(B73)&gt;0,-B135/B73,0)</f>
-        <v>2.5648020658446121E-2</v>
+        <v>2.517589096438734E-2</v>
       </c>
     </row>
     <row r="144" spans="1:5" s="12" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
@@ -76546,7 +76920,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{207BDDBF-6D10-452B-9124-D2C10463CF65}">
-  <dimension ref="A3:L47"/>
+  <dimension ref="A3:L48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.140625" bestFit="1" customWidth="1"/>
@@ -76602,13 +76976,13 @@
         <v>1290.4129487784612</v>
       </c>
       <c r="E4" s="35">
-        <v>13275.558198955154</v>
+        <v>13373.602412485154</v>
       </c>
       <c r="G4" s="35">
-        <v>13275.558198955154</v>
+        <v>13373.602412485154</v>
       </c>
       <c r="J4" s="35">
-        <v>14072.586580620899</v>
+        <v>14173.606984500899</v>
       </c>
       <c r="L4" s="35">
         <v>1163.7736081299997</v>
@@ -76633,27 +77007,27 @@
         <v>32</v>
       </c>
       <c r="B6" s="35">
-        <v>3633.6654573699998</v>
+        <v>3734.68586125</v>
       </c>
       <c r="C6" s="35">
-        <v>2707.9265223937</v>
+        <v>2805.9707359237</v>
       </c>
       <c r="E6" s="36">
         <f>GETPIVOTDATA("Aktuelle Position €",$E$3)</f>
-        <v>13275.558198955154</v>
+        <v>13373.602412485154</v>
       </c>
       <c r="G6" s="36">
         <f>GETPIVOTDATA("Aktuelle Position €",$G$3)</f>
-        <v>13275.558198955154</v>
+        <v>13373.602412485154</v>
       </c>
       <c r="H6" s="36"/>
       <c r="I6" s="36">
         <f>G6-J6</f>
-        <v>-797.02838166574475</v>
+        <v>-800.004572015745</v>
       </c>
       <c r="J6" s="36">
         <f>GETPIVOTDATA("Aktuell Investiert €",$J$3)</f>
-        <v>14072.586580620899</v>
+        <v>14173.606984500899</v>
       </c>
       <c r="L6" s="36">
         <f>GETPIVOTDATA("Realisierte P&amp;L Verkäufe €",$L$3)</f>
@@ -76665,10 +77039,10 @@
         <v>1431</v>
       </c>
       <c r="B7" s="35">
-        <v>14072.586580620899</v>
+        <v>14173.606984500899</v>
       </c>
       <c r="C7" s="35">
-        <v>13275.558198955161</v>
+        <v>13373.602412485161</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -76724,7 +77098,7 @@
         <v>32</v>
       </c>
       <c r="F16" s="35">
-        <v>2707.9265223937</v>
+        <v>2805.9707359237</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -76738,7 +77112,7 @@
         <v>1431</v>
       </c>
       <c r="F17" s="35">
-        <v>13275.558198955161</v>
+        <v>13373.602412485161</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -76906,7 +77280,7 @@
         <v>32</v>
       </c>
       <c r="B38" s="35">
-        <v>2707.9265223937</v>
+        <v>2805.9707359237</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -76974,11 +77348,19 @@
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="9" t="s">
+      <c r="A47" s="34" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B47" s="35">
+        <v>98.044213529999993</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="9" t="s">
         <v>1431</v>
       </c>
-      <c r="B47" s="35">
-        <v>13275.558198955157</v>
+      <c r="B48" s="35">
+        <v>13373.602412485157</v>
       </c>
     </row>
   </sheetData>
@@ -77496,55 +77878,128 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="34" t="s">
+        <v>1444</v>
+      </c>
+      <c r="B46" s="28">
+        <v>8.5034010000000002</v>
+      </c>
+      <c r="C46" s="37">
+        <v>11.53</v>
+      </c>
+      <c r="D46" s="37">
+        <v>98.044213529999993</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
         <v>1439</v>
       </c>
-      <c r="B46" s="28">
-        <v>900.74177199999997</v>
-      </c>
-      <c r="C46" s="37">
-        <v>175.77419999999998</v>
-      </c>
-      <c r="D46" s="37">
-        <v>2707.9265223937</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="9"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="37"/>
-      <c r="D47" s="37"/>
+      <c r="B47" s="28">
+        <v>909.24517300000002</v>
+      </c>
+      <c r="C47" s="37">
+        <v>187.30419999999998</v>
+      </c>
+      <c r="D47" s="37">
+        <v>2805.9707359237</v>
+      </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="9" t="s">
+      <c r="A48" s="9"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="37"/>
+      <c r="D48" s="37"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49" s="9" t="s">
         <v>1431</v>
       </c>
-      <c r="B48" s="28">
-        <v>3881.5755840000002</v>
-      </c>
-      <c r="C48" s="37">
-        <v>2068.7425188984689</v>
-      </c>
-      <c r="D48" s="37">
-        <v>13275.558198955157</v>
-      </c>
-    </row>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+      <c r="B49" s="28">
+        <v>3890.0789850000001</v>
+      </c>
+      <c r="C49" s="37">
+        <v>2080.2725188984691</v>
+      </c>
+      <c r="D49" s="37">
+        <v>13373.602412485157</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B50"/>
+      <c r="C50"/>
+      <c r="D50"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B51"/>
+      <c r="C51"/>
+      <c r="D51"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B52"/>
+      <c r="C52"/>
+      <c r="D52"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B53"/>
+      <c r="C53"/>
+      <c r="D53"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B54"/>
+      <c r="C54"/>
+      <c r="D54"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B55"/>
+      <c r="C55"/>
+      <c r="D55"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B56"/>
+      <c r="C56"/>
+      <c r="D56"/>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B57"/>
+      <c r="C57"/>
+      <c r="D57"/>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B58"/>
+      <c r="C58"/>
+      <c r="D58"/>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B59"/>
+      <c r="C59"/>
+      <c r="D59"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B60"/>
+      <c r="C60"/>
+      <c r="D60"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B61"/>
+      <c r="C61"/>
+      <c r="D61"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B62"/>
+      <c r="C62"/>
+      <c r="D62"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B63"/>
+      <c r="C63"/>
+      <c r="D63"/>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B64"/>
+      <c r="C64"/>
+      <c r="D64"/>
+    </row>
     <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Changes in der formel manuel done
</commit_message>
<xml_diff>
--- a/Auswertung/Portfolio_Profi_Analyse_B.xlsx
+++ b/Auswertung/Portfolio_Profi_Analyse_B.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Documents\Portfolio_Excel\Auswertung\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4109DD9-4038-40F9-AE3C-D830B847161B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{381FDE32-1F23-4745-A108-C383CAF37317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daten" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="14" r:id="rId11"/>
+    <pivotCache cacheId="0" r:id="rId11"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -19477,356 +19477,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8E326F01-EA15-4A93-82D4-848E4D2615C7}" name="PivotTable9" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
-  <location ref="J3:J4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="24">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Einkaufswert" fld="16" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="16">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{223E5646-EA4E-4DBC-8347-0CFCE76D5F19}" name="PivotTable5" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Assets">
-  <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="24">
-    <pivotField showAll="0">
-      <items count="64">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="37"/>
-        <item x="38"/>
-        <item x="39"/>
-        <item x="40"/>
-        <item x="41"/>
-        <item x="42"/>
-        <item x="43"/>
-        <item x="44"/>
-        <item x="45"/>
-        <item x="46"/>
-        <item x="47"/>
-        <item x="48"/>
-        <item x="49"/>
-        <item x="50"/>
-        <item x="51"/>
-        <item x="52"/>
-        <item x="53"/>
-        <item x="54"/>
-        <item x="55"/>
-        <item x="56"/>
-        <item x="57"/>
-        <item x="58"/>
-        <item x="59"/>
-        <item x="60"/>
-        <item x="61"/>
-        <item x="62"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="Einkaufswert" fld="16" baseField="0" baseItem="0"/>
-    <dataField name="Aktueller Wert" fld="15" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="17">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="3" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E0769888-D3D4-498F-9981-49DFC80F5D0F}" name="PivotTable8" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
-  <location ref="G3:G4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="24">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Aktueller Wert" fld="15" baseField="0" baseItem="0" numFmtId="44"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="18">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1A3F31EA-6894-49F2-AD85-69A514AE323F}" name="PivotTable1" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
-  <location ref="L3:L4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="24">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Verkaufserlöse Gewinn/Verlust" fld="18" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="19">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9691FC7-B584-44C9-8056-E4ED1D6024DD}" name="PivotTable11" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E9691FC7-B584-44C9-8056-E4ED1D6024DD}" name="PivotTable11" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
   <location ref="E3:E4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="24">
     <pivotField showAll="0"/>
@@ -19872,7 +19523,7 @@
     <dataField name="Aktueller Wert" fld="15" baseField="0" baseItem="0" numFmtId="44"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="20">
+    <format dxfId="16">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -19888,8 +19539,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D646C2F3-32F0-4399-B83F-C10E1649A49F}" name="PivotTable6" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" preserveFormatting="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="Assets">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D646C2F3-32F0-4399-B83F-C10E1649A49F}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" preserveFormatting="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11" rowHeaderCaption="Assets">
   <location ref="A13:B45" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="24">
     <pivotField axis="axisRow" showAll="0" measureFilter="1">
@@ -21122,8 +20773,239 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4A41211-FADE-4A81-A35B-B4ED20E62223}" name="PivotTable10" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Assets">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8E326F01-EA15-4A93-82D4-848E4D2615C7}" name="PivotTable9" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+  <location ref="J3:J4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="24">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Einkaufswert" fld="16" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="17">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{223E5646-EA4E-4DBC-8347-0CFCE76D5F19}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4" rowHeaderCaption="Assets">
+  <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="24">
+    <pivotField showAll="0">
+      <items count="64">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item x="50"/>
+        <item x="51"/>
+        <item x="52"/>
+        <item x="53"/>
+        <item x="54"/>
+        <item x="55"/>
+        <item x="56"/>
+        <item x="57"/>
+        <item x="58"/>
+        <item x="59"/>
+        <item x="60"/>
+        <item x="61"/>
+        <item x="62"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="Einkaufswert" fld="16" baseField="0" baseItem="0"/>
+    <dataField name="Aktueller Wert" fld="15" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="18">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="3" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D4A41211-FADE-4A81-A35B-B4ED20E62223}" name="PivotTable10" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5" rowHeaderCaption="Assets">
   <location ref="E13:F18" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="24">
     <pivotField showAll="0">
@@ -21253,7 +21135,7 @@
     <dataField name="Aktueller Wert" fld="15" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="21">
+    <format dxfId="19">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
   </formats>
@@ -21328,8 +21210,126 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E0769888-D3D4-498F-9981-49DFC80F5D0F}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+  <location ref="G3:G4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="24">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Aktueller Wert" fld="15" baseField="0" baseItem="0" numFmtId="44"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="20">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1A3F31EA-6894-49F2-AD85-69A514AE323F}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+  <location ref="L3:L4" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="24">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Verkaufserlöse Gewinn/Verlust" fld="18" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="21">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{745C1A6C-3C9D-40E8-BB3C-38468AC3798B}" name="PivotTable12" cacheId="14" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{745C1A6C-3C9D-40E8-BB3C-38468AC3798B}" name="PivotTable12" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Werte" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Assets">
   <location ref="A8:D46" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="24">
     <pivotField axis="axisRow" subtotalTop="0" showAll="0" insertBlankRow="1" measureFilter="1">
@@ -71955,7 +71955,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="6">
-        <f>IF(E2&gt;0,E2+F2-D2,0)</f>
+        <f>IF(E2&gt;0,E2+G2-D2,0)</f>
         <v>0</v>
       </c>
     </row>
@@ -71986,8 +71986,8 @@
         <v>3</v>
       </c>
       <c r="H3" s="6">
-        <f>IF(E3&gt;0,E3+F3-D3,0)</f>
-        <v>546.02</v>
+        <f t="shared" ref="H3:H63" si="0">IF(E3&gt;0,E3+G3-D3,0)</f>
+        <v>544.02</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -72017,8 +72017,8 @@
         <v>3</v>
       </c>
       <c r="H4" s="6">
-        <f t="shared" ref="H3:H63" si="0">IF(E4&gt;0,E4+F4-D4,0)</f>
-        <v>654.62</v>
+        <f t="shared" si="0"/>
+        <v>653.62</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -72049,7 +72049,7 @@
       </c>
       <c r="H5" s="6">
         <f t="shared" si="0"/>
-        <v>649.99</v>
+        <v>638.99</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -72080,7 +72080,7 @@
       </c>
       <c r="H6" s="6">
         <f t="shared" si="0"/>
-        <v>249.99999999999997</v>
+        <v>248.99999999999997</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -72142,7 +72142,7 @@
       </c>
       <c r="H8" s="6">
         <f t="shared" si="0"/>
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -72173,7 +72173,7 @@
       </c>
       <c r="H9" s="6">
         <f t="shared" si="0"/>
-        <v>253.99999999999997</v>
+        <v>247.99999999999997</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -72235,7 +72235,7 @@
       </c>
       <c r="H11" s="6">
         <f t="shared" si="0"/>
-        <v>1083.74</v>
+        <v>1078.74</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -72266,7 +72266,7 @@
       </c>
       <c r="H12" s="6">
         <f t="shared" si="0"/>
-        <v>996.12999999999988</v>
+        <v>990.12999999999988</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -72328,7 +72328,7 @@
       </c>
       <c r="H14" s="6">
         <f t="shared" si="0"/>
-        <v>505.08000000000004</v>
+        <v>504.08000000000004</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -72514,7 +72514,7 @@
       </c>
       <c r="H20" s="6">
         <f t="shared" si="0"/>
-        <v>1470.1</v>
+        <v>1447.1</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -72545,7 +72545,7 @@
       </c>
       <c r="H21" s="6">
         <f t="shared" si="0"/>
-        <v>1888.21</v>
+        <v>1874.21</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -72576,7 +72576,7 @@
       </c>
       <c r="H22" s="6">
         <f t="shared" si="0"/>
-        <v>355.01000000000005</v>
+        <v>354.01000000000005</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -72638,7 +72638,7 @@
       </c>
       <c r="H24" s="6">
         <f t="shared" si="0"/>
-        <v>91.71</v>
+        <v>92.71</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -72700,7 +72700,7 @@
       </c>
       <c r="H26" s="6">
         <f t="shared" si="0"/>
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -72762,7 +72762,7 @@
       </c>
       <c r="H28" s="6">
         <f t="shared" si="0"/>
-        <v>260.54000000000002</v>
+        <v>258.54000000000002</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -73010,7 +73010,7 @@
       </c>
       <c r="H36" s="6">
         <f t="shared" si="0"/>
-        <v>606.00999999999988</v>
+        <v>605.00999999999988</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -73072,7 +73072,7 @@
       </c>
       <c r="H38" s="6">
         <f t="shared" si="0"/>
-        <v>275.99</v>
+        <v>272.99</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -73413,7 +73413,7 @@
       </c>
       <c r="H49" s="6">
         <f t="shared" si="0"/>
-        <v>79.8</v>
+        <v>80.8</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -73444,7 +73444,7 @@
       </c>
       <c r="H50" s="6">
         <f t="shared" si="0"/>
-        <v>1077.26</v>
+        <v>1071.26</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -73506,7 +73506,7 @@
       </c>
       <c r="H52" s="6">
         <f t="shared" si="0"/>
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -73568,7 +73568,7 @@
       </c>
       <c r="H54" s="6">
         <f t="shared" si="0"/>
-        <v>117.99</v>
+        <v>118.99</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -73630,7 +73630,7 @@
       </c>
       <c r="H56" s="6">
         <f t="shared" si="0"/>
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -74055,9 +74055,9 @@
         <v>0</v>
       </c>
       <c r="T2" s="6">
-        <f t="shared" ref="T2:T33" si="6">IF(E2=0,
+        <f>IF(E2=0,
 0,
-(G2-(F2*M2))+I2
+(G2-(F2*M2))+V2
 )</f>
         <v>0</v>
       </c>
@@ -74121,7 +74121,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="6">
-        <f t="shared" ref="K3:K63" si="7">H3-G3-I3-J3</f>
+        <f t="shared" ref="K3:K63" si="6">H3-G3-I3-J3</f>
         <v>96.949999999999932</v>
       </c>
       <c r="L3" s="5" t="str">
@@ -74162,7 +74162,10 @@
         <v>117.1472252399999</v>
       </c>
       <c r="T3" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="T3:T33" si="7">IF(E3=0,
+0,
+(G3-(F3*M3))+I3
+)</f>
         <v>544.38277476000007</v>
       </c>
       <c r="U3" s="26">
@@ -74225,7 +74228,7 @@
         <v>0</v>
       </c>
       <c r="K4" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>27.860000000000014</v>
       </c>
       <c r="L4" s="5" t="str">
@@ -74266,7 +74269,7 @@
         <v>31.260000000000012</v>
       </c>
       <c r="T4" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>657</v>
       </c>
       <c r="U4" s="26">
@@ -74329,7 +74332,7 @@
         <v>0</v>
       </c>
       <c r="K5" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>88.029999999999973</v>
       </c>
       <c r="L5" s="5" t="str">
@@ -74370,7 +74373,7 @@
         <v>88.029999999999973</v>
       </c>
       <c r="T5" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>639</v>
       </c>
       <c r="U5" s="26">
@@ -74429,7 +74432,7 @@
         <v>0</v>
       </c>
       <c r="K6" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-6.5400000000000205</v>
       </c>
       <c r="L6" s="5" t="str">
@@ -74470,7 +74473,7 @@
         <v>-6.5400000000000205</v>
       </c>
       <c r="T6" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>249</v>
       </c>
       <c r="U6" s="26">
@@ -74529,7 +74532,7 @@
         <v>0</v>
       </c>
       <c r="K7" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-183.99</v>
       </c>
       <c r="L7" s="5" t="str">
@@ -74570,7 +74573,7 @@
         <v>0</v>
       </c>
       <c r="T7" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U7" s="26">
@@ -74629,7 +74632,7 @@
         <v>0</v>
       </c>
       <c r="K8" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>50.620000000000005</v>
       </c>
       <c r="L8" s="5" t="str">
@@ -74670,7 +74673,7 @@
         <v>50.620000000000005</v>
       </c>
       <c r="T8" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>202</v>
       </c>
       <c r="U8" s="26">
@@ -74729,7 +74732,7 @@
         <v>0</v>
       </c>
       <c r="K9" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-167.09000000000003</v>
       </c>
       <c r="L9" s="5" t="str">
@@ -74770,7 +74773,7 @@
         <v>14.501886909999939</v>
       </c>
       <c r="T9" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>249.02811309000003</v>
       </c>
       <c r="U9" s="26">
@@ -74829,7 +74832,7 @@
         <v>0</v>
       </c>
       <c r="K10" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-699.08</v>
       </c>
       <c r="L10" s="5" t="str">
@@ -74870,7 +74873,7 @@
         <v>0</v>
       </c>
       <c r="T10" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U10" s="26">
@@ -74929,7 +74932,7 @@
         <v>16.5</v>
       </c>
       <c r="K11" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>104.41000000000008</v>
       </c>
       <c r="L11" s="5" t="str">
@@ -74970,7 +74973,7 @@
         <v>120.91000000000008</v>
       </c>
       <c r="T11" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1058.99</v>
       </c>
       <c r="U11" s="26">
@@ -75029,7 +75032,7 @@
         <v>13.16</v>
       </c>
       <c r="K12" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-727.04000000000008</v>
       </c>
       <c r="L12" s="5" t="str">
@@ -75070,7 +75073,7 @@
         <v>186.75221787000021</v>
       </c>
       <c r="T12" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>947.24778212999979</v>
       </c>
       <c r="U12" s="26">
@@ -75129,7 +75132,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-706.81</v>
       </c>
       <c r="L13" s="5" t="str">
@@ -75170,7 +75173,7 @@
         <v>0</v>
       </c>
       <c r="T13" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U13" s="26">
@@ -75229,7 +75232,7 @@
         <v>0</v>
       </c>
       <c r="K14" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>3.6100000000000136</v>
       </c>
       <c r="L14" s="5" t="str">
@@ -75270,7 +75273,7 @@
         <v>3.6100000000000136</v>
       </c>
       <c r="T14" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>503</v>
       </c>
       <c r="U14" s="26">
@@ -75329,7 +75332,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-402.98999999999995</v>
       </c>
       <c r="L15" s="5" t="str">
@@ -75370,7 +75373,7 @@
         <v>0</v>
       </c>
       <c r="T15" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U15" s="26">
@@ -75429,7 +75432,7 @@
         <v>0</v>
       </c>
       <c r="K16" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-57.55</v>
       </c>
       <c r="L16" s="5" t="str">
@@ -75470,7 +75473,7 @@
         <v>0</v>
       </c>
       <c r="T16" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U16" s="26">
@@ -75529,7 +75532,7 @@
         <v>0</v>
       </c>
       <c r="K17" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-101</v>
       </c>
       <c r="L17" s="5" t="str">
@@ -75570,7 +75573,7 @@
         <v>0</v>
       </c>
       <c r="T17" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U17" s="26">
@@ -75629,7 +75632,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>41.97</v>
       </c>
       <c r="L18" s="5" t="str">
@@ -75670,7 +75673,7 @@
         <v>41.97</v>
       </c>
       <c r="T18" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>81</v>
       </c>
       <c r="U18" s="26">
@@ -75729,7 +75732,7 @@
         <v>0</v>
       </c>
       <c r="K19" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-657.91</v>
       </c>
       <c r="L19" s="5" t="str">
@@ -75770,7 +75773,7 @@
         <v>0</v>
       </c>
       <c r="T19" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U19" s="26">
@@ -75829,7 +75832,7 @@
         <v>40.070000000000007</v>
       </c>
       <c r="K20" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-1247.9599999999994</v>
       </c>
       <c r="L20" s="5" t="str">
@@ -75870,7 +75873,7 @@
         <v>229.91123263200052</v>
       </c>
       <c r="T20" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1486.7087673679994</v>
       </c>
       <c r="U20" s="26">
@@ -75929,7 +75932,7 @@
         <v>15.58</v>
       </c>
       <c r="K21" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-595.35000000000048</v>
       </c>
       <c r="L21" s="5" t="str">
@@ -75970,7 +75973,7 @@
         <v>228.55568621999964</v>
       </c>
       <c r="T21" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1890.0143137800001</v>
       </c>
       <c r="U21" s="26">
@@ -76029,7 +76032,7 @@
         <v>0</v>
       </c>
       <c r="K22" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>17.710000000000036</v>
       </c>
       <c r="L22" s="5" t="str">
@@ -76070,7 +76073,7 @@
         <v>17.710000000000036</v>
       </c>
       <c r="T22" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>354</v>
       </c>
       <c r="U22" s="26">
@@ -76129,7 +76132,7 @@
         <v>0</v>
       </c>
       <c r="K23" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>18.149999999999991</v>
       </c>
       <c r="L23" s="5" t="str">
@@ -76170,7 +76173,7 @@
         <v>18.149999999999991</v>
       </c>
       <c r="T23" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>101</v>
       </c>
       <c r="U23" s="26">
@@ -76229,7 +76232,7 @@
         <v>2.29</v>
       </c>
       <c r="K24" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>6.4100000000000028</v>
       </c>
       <c r="L24" s="5" t="str">
@@ -76270,7 +76273,7 @@
         <v>8.7000000000000028</v>
       </c>
       <c r="T24" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>95</v>
       </c>
       <c r="U24" s="26">
@@ -76329,7 +76332,7 @@
         <v>0.57000000000000006</v>
       </c>
       <c r="K25" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1.5899999999999965</v>
       </c>
       <c r="L25" s="5" t="str">
@@ -76370,7 +76373,7 @@
         <v>2.1599999999999966</v>
       </c>
       <c r="T25" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>62</v>
       </c>
       <c r="U25" s="26">
@@ -76429,7 +76432,7 @@
         <v>0</v>
       </c>
       <c r="K26" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-348.69000000000005</v>
       </c>
       <c r="L26" s="5" t="str">
@@ -76470,7 +76473,7 @@
         <v>8.1364286399999912</v>
       </c>
       <c r="T26" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>202.13357136000002</v>
       </c>
       <c r="U26" s="26">
@@ -76529,7 +76532,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>15.349999999999994</v>
       </c>
       <c r="L27" s="5" t="str">
@@ -76570,7 +76573,7 @@
         <v>15.349999999999994</v>
       </c>
       <c r="T27" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>101</v>
       </c>
       <c r="U27" s="26">
@@ -76629,7 +76632,7 @@
         <v>12.07</v>
       </c>
       <c r="K28" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-466.64</v>
       </c>
       <c r="L28" s="5" t="str">
@@ -76670,7 +76673,7 @@
         <v>65.430000000000007</v>
       </c>
       <c r="T28" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>250.99</v>
       </c>
       <c r="U28" s="26">
@@ -76729,7 +76732,7 @@
         <v>0</v>
       </c>
       <c r="K29" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-400.96</v>
       </c>
       <c r="L29" s="5" t="str">
@@ -76770,7 +76773,7 @@
         <v>0</v>
       </c>
       <c r="T29" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U29" s="26">
@@ -76829,7 +76832,7 @@
         <v>0</v>
       </c>
       <c r="K30" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-551</v>
       </c>
       <c r="L30" s="5" t="str">
@@ -76870,7 +76873,7 @@
         <v>0</v>
       </c>
       <c r="T30" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U30" s="26">
@@ -76929,7 +76932,7 @@
         <v>0</v>
       </c>
       <c r="K31" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-533.53</v>
       </c>
       <c r="L31" s="5" t="str">
@@ -76970,7 +76973,7 @@
         <v>0</v>
       </c>
       <c r="T31" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U31" s="26">
@@ -77029,7 +77032,7 @@
         <v>0</v>
       </c>
       <c r="K32" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-403.01</v>
       </c>
       <c r="L32" s="5" t="str">
@@ -77070,7 +77073,7 @@
         <v>0</v>
       </c>
       <c r="T32" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U32" s="26">
@@ -77129,7 +77132,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-271.15999999999997</v>
       </c>
       <c r="L33" s="5" t="str">
@@ -77170,7 +77173,7 @@
         <v>0</v>
       </c>
       <c r="T33" s="6">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="U33" s="26">
@@ -77229,7 +77232,7 @@
         <v>1.6</v>
       </c>
       <c r="K34" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>3.5899999999999976</v>
       </c>
       <c r="L34" s="5" t="str">
@@ -77339,7 +77342,7 @@
         <v>2.7600000000000002</v>
       </c>
       <c r="K35" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>7.74</v>
       </c>
       <c r="L35" s="5" t="str">
@@ -77439,7 +77442,7 @@
         <v>0</v>
       </c>
       <c r="K36" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>28.099999999999909</v>
       </c>
       <c r="L36" s="5" t="str">
@@ -77539,7 +77542,7 @@
         <v>0</v>
       </c>
       <c r="K37" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0.27000000000001023</v>
       </c>
       <c r="L37" s="5" t="str">
@@ -77639,7 +77642,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>6.4499999999999886</v>
       </c>
       <c r="L38" s="5" t="str">
@@ -77739,7 +77742,7 @@
         <v>0</v>
       </c>
       <c r="K39" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-117.99</v>
       </c>
       <c r="L39" s="5" t="str">
@@ -77839,7 +77842,7 @@
         <v>0</v>
       </c>
       <c r="K40" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-24</v>
       </c>
       <c r="L40" s="5" t="str">
@@ -77939,7 +77942,7 @@
         <v>0</v>
       </c>
       <c r="K41" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-402.95</v>
       </c>
       <c r="L41" s="5" t="str">
@@ -78039,7 +78042,7 @@
         <v>0</v>
       </c>
       <c r="K42" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>17.839999999999989</v>
       </c>
       <c r="L42" s="5" t="str">
@@ -78139,7 +78142,7 @@
         <v>0</v>
       </c>
       <c r="K43" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>44.790000000000006</v>
       </c>
       <c r="L43" s="5" t="str">
@@ -78239,7 +78242,7 @@
         <v>0</v>
       </c>
       <c r="K44" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-58.97</v>
       </c>
       <c r="L44" s="5" t="str">
@@ -78339,7 +78342,7 @@
         <v>1.92</v>
       </c>
       <c r="K45" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>5.3600000000000012</v>
       </c>
       <c r="L45" s="5" t="str">
@@ -78439,7 +78442,7 @@
         <v>0.64</v>
       </c>
       <c r="K46" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1.8299999999999987</v>
       </c>
       <c r="L46" s="5" t="str">
@@ -78539,7 +78542,7 @@
         <v>10.210000000000001</v>
       </c>
       <c r="K47" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>48.87000000000004</v>
       </c>
       <c r="L47" s="5" t="str">
@@ -78639,7 +78642,7 @@
         <v>2.16</v>
       </c>
       <c r="K48" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>6.0299999999999976</v>
       </c>
       <c r="L48" s="5" t="str">
@@ -78739,7 +78742,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="K49" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>7.1000000000000112</v>
       </c>
       <c r="L49" s="5" t="str">
@@ -78839,7 +78842,7 @@
         <v>0</v>
       </c>
       <c r="K50" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>74.259999999999991</v>
       </c>
       <c r="L50" s="5" t="str">
@@ -78939,7 +78942,7 @@
         <v>0</v>
       </c>
       <c r="K51" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-607.06000000000006</v>
       </c>
       <c r="L51" s="5" t="str">
@@ -79039,7 +79042,7 @@
         <v>0</v>
       </c>
       <c r="K52" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>6.5</v>
       </c>
       <c r="L52" s="5" t="str">
@@ -79139,7 +79142,7 @@
         <v>0.37</v>
       </c>
       <c r="K53" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1.0700000000000012</v>
       </c>
       <c r="L53" s="5" t="str">
@@ -79239,7 +79242,7 @@
         <v>0</v>
       </c>
       <c r="K54" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-17.850000000000009</v>
       </c>
       <c r="L54" s="5" t="str">
@@ -79339,7 +79342,7 @@
         <v>0</v>
       </c>
       <c r="K55" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-833.58000000000015</v>
       </c>
       <c r="L55" s="5" t="str">
@@ -79439,7 +79442,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>78.63</v>
       </c>
       <c r="L56" s="5" t="str">
@@ -79539,7 +79542,7 @@
         <v>0</v>
       </c>
       <c r="K57" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>1.3000000000000007</v>
       </c>
       <c r="L57" s="5" t="str">
@@ -79639,7 +79642,7 @@
         <v>0</v>
       </c>
       <c r="K58" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>10.629999999999995</v>
       </c>
       <c r="L58" s="5" t="str">
@@ -79739,7 +79742,7 @@
         <v>0</v>
       </c>
       <c r="K59" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>3.1599999999999966</v>
       </c>
       <c r="L59" s="5" t="str">
@@ -79839,7 +79842,7 @@
         <v>0</v>
       </c>
       <c r="K60" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>19.329999999999984</v>
       </c>
       <c r="L60" s="5" t="str">
@@ -79939,7 +79942,7 @@
         <v>0</v>
       </c>
       <c r="K61" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0.31000000000000227</v>
       </c>
       <c r="L61" s="5" t="str">
@@ -80039,7 +80042,7 @@
         <v>0</v>
       </c>
       <c r="K62" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-312.45</v>
       </c>
       <c r="L62" s="5" t="str">
@@ -80139,7 +80142,7 @@
         <v>0</v>
       </c>
       <c r="K63" s="6">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>-101</v>
       </c>
       <c r="L63" s="5" t="str">

</xml_diff>